<commit_message>
Update demo Excel: fix column headers to match system mapping
</commit_message>
<xml_diff>
--- a/public/emergency/demo_residents.xlsx
+++ b/public/emergency/demo_residents.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>ת.ז.</t>
+          <t>ת"ז</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>מרכז משפחתי</t>
+          <t>מרכז משפחות</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
@@ -644,7 +644,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>מרכז קהילתי רמת יוסף</t>
+          <t>מרכז משפחות רמת יוסף</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr"/>
@@ -696,7 +696,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>מרכז קהילתי רמת יוסף</t>
+          <t>מרכז משפחות רמת יוסף</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr"/>
@@ -804,7 +804,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי צפון</t>
+          <t>מרכז משפחות צפון</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי רמת יוסף</t>
+          <t>מרכז משפחות רמת יוסף</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
@@ -968,7 +968,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr"/>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי צפון</t>
+          <t>מרכז משפחות צפון</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>מרכז קהילתי רמת יוסף</t>
+          <t>מרכז משפחות רמת יוסף</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr"/>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>מרכז קהילתי צפון</t>
+          <t>מרכז משפחות צפון</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי צפון</t>
+          <t>מרכז משפחות צפון</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr"/>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>מרכז קהילתי רמת יוסף</t>
+          <t>מרכז משפחות רמת יוסף</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr"/>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי צפון</t>
+          <t>מרכז משפחות צפון</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr"/>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>מרכז קהילתי רמת יוסף</t>
+          <t>מרכז משפחות רמת יוסף</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr"/>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>מרכז קהילתי צפון</t>
+          <t>מרכז משפחות צפון</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr"/>
@@ -1662,7 +1662,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>מרכז קהילתי גאולה</t>
+          <t>מרכז משפחות גאולה</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1688,7 +1688,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>מרכז קהילתי רמת יוסף</t>
+          <t>מרכז משפחות רמת יוסף</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -1714,7 +1714,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>מרכז קהילתי צפון</t>
+          <t>מרכז משפחות צפון</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">

</xml_diff>